<commit_message>
feat: enable multiple selection for Agencia filter in bandeja
</commit_message>
<xml_diff>
--- a/CONVENIOS.xlsx
+++ b/CONVENIOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CRM PYP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80804BD8-8E73-4E7A-9626-37540BB909A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C2FCEF1-3B74-4AC3-9233-68D75C1E4F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{ECA4CCC5-1254-447A-8251-91EACE3DDB72}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="207">
   <si>
     <t>Agencia</t>
   </si>
@@ -73,9 +73,6 @@
     <t>013</t>
   </si>
   <si>
-    <t>2026.07.11</t>
-  </si>
-  <si>
     <t>NO</t>
   </si>
   <si>
@@ -88,9 +85,6 @@
     <t>-</t>
   </si>
   <si>
-    <t>2026.07.14</t>
-  </si>
-  <si>
     <t>107038101002466200</t>
   </si>
   <si>
@@ -100,9 +94,6 @@
     <t>002</t>
   </si>
   <si>
-    <t>2026.07.29</t>
-  </si>
-  <si>
     <t>SI</t>
   </si>
   <si>
@@ -118,9 +109,6 @@
     <t>012</t>
   </si>
   <si>
-    <t>2026.07.09</t>
-  </si>
-  <si>
     <t>107038101001307784</t>
   </si>
   <si>
@@ -130,9 +118,6 @@
     <t>008</t>
   </si>
   <si>
-    <t>2026.07.26</t>
-  </si>
-  <si>
     <t>107038101002997988</t>
   </si>
   <si>
@@ -142,12 +127,6 @@
     <t>003</t>
   </si>
   <si>
-    <t>2026.08.18</t>
-  </si>
-  <si>
-    <t>2025.12.30</t>
-  </si>
-  <si>
     <t>107038101002180423</t>
   </si>
   <si>
@@ -157,12 +136,6 @@
     <t>001</t>
   </si>
   <si>
-    <t>2025.08.25</t>
-  </si>
-  <si>
-    <t>2026.06.16</t>
-  </si>
-  <si>
     <t>107038101002924413</t>
   </si>
   <si>
@@ -172,36 +145,24 @@
     <t>INVERSIONES CRISTELLE AD E.I.R.L.</t>
   </si>
   <si>
-    <t>2026.07.28</t>
-  </si>
-  <si>
     <t>107038101002204929</t>
   </si>
   <si>
     <t>MORALES SANCHEZ, DANY DANIEL</t>
   </si>
   <si>
-    <t>2025.08.28</t>
-  </si>
-  <si>
     <t>107038101002365202</t>
   </si>
   <si>
     <t>PORROA SAAVEDRA, BETTSY KATERINE</t>
   </si>
   <si>
-    <t>2026.07.30</t>
-  </si>
-  <si>
     <t>107038101002761400</t>
   </si>
   <si>
     <t>SERVICIOS INTEGRALES GALINDO S.A.C</t>
   </si>
   <si>
-    <t>2026.07.23</t>
-  </si>
-  <si>
     <t>107038101002139328</t>
   </si>
   <si>
@@ -214,9 +175,6 @@
     <t>CASTILLO HUAMAN VDA DE FLORES, OLGA JUVENCIA</t>
   </si>
   <si>
-    <t>2026.07.25</t>
-  </si>
-  <si>
     <t>107038101003343467</t>
   </si>
   <si>
@@ -226,9 +184,6 @@
     <t>011</t>
   </si>
   <si>
-    <t>2026.07.22</t>
-  </si>
-  <si>
     <t>AG. SURQUILLO</t>
   </si>
   <si>
@@ -238,9 +193,6 @@
     <t>HUARHUA VELA, FLOR DE MARIA</t>
   </si>
   <si>
-    <t>2026.08.13</t>
-  </si>
-  <si>
     <t>107024101005795370</t>
   </si>
   <si>
@@ -262,9 +214,6 @@
     <t>ALANYA VELASQUEZ, ROGER GERMAN</t>
   </si>
   <si>
-    <t>2025.03.30</t>
-  </si>
-  <si>
     <t>107074101001393345</t>
   </si>
   <si>
@@ -280,18 +229,12 @@
     <t>009</t>
   </si>
   <si>
-    <t>2026.08.24</t>
-  </si>
-  <si>
     <t>107074101000996919</t>
   </si>
   <si>
     <t>AGUILAR TORRES, MARIA DEL CARMEN</t>
   </si>
   <si>
-    <t>2026.07.24</t>
-  </si>
-  <si>
     <t>107074101001608015</t>
   </si>
   <si>
@@ -304,9 +247,6 @@
     <t>CORPORACION SANCHEZ H S.A.C.</t>
   </si>
   <si>
-    <t>2025.04.11</t>
-  </si>
-  <si>
     <t>107074101001973375</t>
   </si>
   <si>
@@ -325,9 +265,6 @@
     <t>NEVERLAN IMPORT E.I.R.L.</t>
   </si>
   <si>
-    <t>2026.08.05</t>
-  </si>
-  <si>
     <t>107074101002048448</t>
   </si>
   <si>
@@ -352,36 +289,24 @@
     <t>007</t>
   </si>
   <si>
-    <t>2026.07.19</t>
-  </si>
-  <si>
     <t>107074101001510031</t>
   </si>
   <si>
     <t>DELGADO CARRERA, GIANCARLO RENZO</t>
   </si>
   <si>
-    <t>2026.08.02</t>
-  </si>
-  <si>
     <t>107074101001983841</t>
   </si>
   <si>
     <t>EGUSQUIZA MEDINA, SARA NOEMI</t>
   </si>
   <si>
-    <t>2026.07.20</t>
-  </si>
-  <si>
     <t>107024101005602791</t>
   </si>
   <si>
     <t>SALAZAR REYNOSO, KAREN MARIELENA</t>
   </si>
   <si>
-    <t>2026.08.15</t>
-  </si>
-  <si>
     <t>AG. CHORRILLOS</t>
   </si>
   <si>
@@ -397,9 +322,6 @@
     <t>LOPEZ MEZA, JUAN CARLOS</t>
   </si>
   <si>
-    <t>2026.02.07</t>
-  </si>
-  <si>
     <t>107099101000734231</t>
   </si>
   <si>
@@ -412,18 +334,12 @@
     <t>INOÑAN REYES, JIMMY ARTURO</t>
   </si>
   <si>
-    <t>2026.06.19</t>
-  </si>
-  <si>
     <t>107099101001382366</t>
   </si>
   <si>
     <t>K &amp; P MAQUINARIAS S.A.C</t>
   </si>
   <si>
-    <t>2026.04.24</t>
-  </si>
-  <si>
     <t>107099101002118170</t>
   </si>
   <si>
@@ -469,18 +385,12 @@
     <t>CHIPANA CRISTOBAL VDA DE CRUZ, IRENE PELAYA</t>
   </si>
   <si>
-    <t>2025.12.28</t>
-  </si>
-  <si>
     <t>107146101001159325</t>
   </si>
   <si>
     <t>FM FRIMARQ CONSTRUCCIONES S.A.C.</t>
   </si>
   <si>
-    <t>2026.07.16</t>
-  </si>
-  <si>
     <t>AG. SAN BORJA</t>
   </si>
   <si>
@@ -493,24 +403,15 @@
     <t>VERGARA SURCO, YRENE</t>
   </si>
   <si>
-    <t>2026.01.23</t>
-  </si>
-  <si>
     <t>107147101000616654</t>
   </si>
   <si>
-    <t>2026.07.05</t>
-  </si>
-  <si>
     <t>107147101000732708</t>
   </si>
   <si>
     <t>VALLADARES VILLALBA, NANCY</t>
   </si>
   <si>
-    <t>2026.10.16</t>
-  </si>
-  <si>
     <t>107147101000210969</t>
   </si>
   <si>
@@ -523,18 +424,12 @@
     <t>ESENARRO SEGURA, ROXANA CRISOLOGA</t>
   </si>
   <si>
-    <t>2026.08.17</t>
-  </si>
-  <si>
     <t>107147101000229395</t>
   </si>
   <si>
     <t>MENDOZA SALCEDO, APRIL MILUSKA</t>
   </si>
   <si>
-    <t>2025.11.30</t>
-  </si>
-  <si>
     <t>AG. SAN GABRIEL</t>
   </si>
   <si>
@@ -583,9 +478,6 @@
     <t>PAJUELO SOTO, AURIA</t>
   </si>
   <si>
-    <t>2026.06.28</t>
-  </si>
-  <si>
     <t>AG. SAN JUAN DE MIRAFLORES II</t>
   </si>
   <si>
@@ -616,9 +508,6 @@
     <t>FINQUIN MENDEZ, MARGOT JANET</t>
   </si>
   <si>
-    <t>2026.08.29</t>
-  </si>
-  <si>
     <t>107178101001012449</t>
   </si>
   <si>
@@ -643,27 +532,18 @@
     <t>BRITO PEREZ, MARIA DE JESUS</t>
   </si>
   <si>
-    <t>2026.07.27</t>
-  </si>
-  <si>
     <t>107178101000591761</t>
   </si>
   <si>
     <t>LLACCTA ZELA, BIVIANA</t>
   </si>
   <si>
-    <t>2026.08.11</t>
-  </si>
-  <si>
     <t>107178101000402160</t>
   </si>
   <si>
     <t>MAMANI SOTO, ORTENCIA</t>
   </si>
   <si>
-    <t>2026.07.31</t>
-  </si>
-  <si>
     <t>107178101000764040</t>
   </si>
   <si>
@@ -676,9 +556,6 @@
     <t>SUMAQ ASOCIADOS SAC</t>
   </si>
   <si>
-    <t>2026.08.09</t>
-  </si>
-  <si>
     <t>AG. LINCE</t>
   </si>
   <si>
@@ -700,9 +577,6 @@
     <t>MINIMARKET EL MERCADER S.A.C</t>
   </si>
   <si>
-    <t>2026.08.10</t>
-  </si>
-  <si>
     <t>107180101000363808</t>
   </si>
   <si>
@@ -730,9 +604,6 @@
     <t>VILLARREAL APAZA, FATIMA RUTH</t>
   </si>
   <si>
-    <t>2026.03.27</t>
-  </si>
-  <si>
     <t>107180101000044541</t>
   </si>
   <si>
@@ -745,9 +616,6 @@
     <t>MENA RAMIREZ, MARCO ANTONIO</t>
   </si>
   <si>
-    <t>2025.10.15</t>
-  </si>
-  <si>
     <t>107180101000325880</t>
   </si>
   <si>
@@ -773,6 +641,9 @@
   </si>
   <si>
     <t>INCA ZAMORA, GLADYS GABRIELA</t>
+  </si>
+  <si>
+    <t>si</t>
   </si>
 </sst>
 </file>
@@ -847,7 +718,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -868,6 +739,9 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1262,28 +1136,28 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>236</v>
+        <v>193</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>237</v>
+        <v>194</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E2" s="10">
         <v>12</v>
       </c>
-      <c r="F2" s="10" t="s">
-        <v>166</v>
+      <c r="F2" s="11">
+        <v>46251</v>
       </c>
       <c r="G2" s="10">
         <v>10</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I2" s="10">
         <v>0</v>
@@ -1295,7 +1169,7 @@
         <v>46221</v>
       </c>
       <c r="L2" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="72.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1303,25 +1177,25 @@
         <v>12</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E3" s="10">
         <v>12</v>
       </c>
-      <c r="F3" s="10" t="s">
-        <v>39</v>
+      <c r="F3" s="11">
+        <v>46252</v>
       </c>
       <c r="G3" s="10">
         <v>999.97</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I3" s="10">
         <v>0</v>
@@ -1333,33 +1207,33 @@
         <v>46220</v>
       </c>
       <c r="L3" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>164</v>
+        <v>131</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>165</v>
+        <v>132</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E4" s="10">
         <v>12</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>166</v>
+      <c r="F4" s="11">
+        <v>46251</v>
       </c>
       <c r="G4" s="10">
         <v>20</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I4" s="10">
         <v>0</v>
@@ -1371,7 +1245,7 @@
         <v>46220</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.15">
@@ -1379,25 +1253,25 @@
         <v>12</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E5" s="10">
         <v>12</v>
       </c>
-      <c r="F5" s="10" t="s">
-        <v>31</v>
+      <c r="F5" s="11">
+        <v>46212</v>
       </c>
       <c r="G5" s="10">
         <v>21163.18</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I5" s="10">
         <v>9</v>
@@ -1409,33 +1283,33 @@
         <v>46219</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>196</v>
+        <v>160</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E6" s="10">
         <v>12</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>197</v>
+      <c r="F6" s="11">
+        <v>46263</v>
       </c>
       <c r="G6" s="10">
         <v>1375.85</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I6" s="10">
         <v>0</v>
@@ -1447,33 +1321,33 @@
         <v>46219</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E7" s="10">
         <v>12</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>118</v>
+      <c r="F7" s="11">
+        <v>46249</v>
       </c>
       <c r="G7" s="10">
         <v>1399.84</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I7" s="10">
         <v>0</v>
@@ -1485,33 +1359,33 @@
         <v>46218</v>
       </c>
       <c r="L7" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>143</v>
+        <v>115</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>144</v>
+        <v>116</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="E8" s="10">
         <v>12</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>118</v>
+      <c r="F8" s="11">
+        <v>46249</v>
       </c>
       <c r="G8" s="10">
         <v>300</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I8" s="10">
         <v>0</v>
@@ -1523,33 +1397,33 @@
         <v>46218</v>
       </c>
       <c r="L8" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>223</v>
+        <v>182</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>224</v>
+        <v>183</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="E9" s="10">
         <v>12</v>
       </c>
-      <c r="F9" s="10" t="s">
-        <v>225</v>
+      <c r="F9" s="11">
+        <v>46244</v>
       </c>
       <c r="G9" s="10">
         <v>999.94</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I9" s="10">
         <v>0</v>
@@ -1561,33 +1435,33 @@
         <v>46214</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A10" s="10" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>221</v>
+        <v>180</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>222</v>
+        <v>181</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E10" s="10">
         <v>12</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>209</v>
+      <c r="F10" s="11">
+        <v>46245</v>
       </c>
       <c r="G10" s="10">
         <v>999.92</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I10" s="10">
         <v>0</v>
@@ -1599,33 +1473,33 @@
         <v>46213</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A11" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>207</v>
+        <v>169</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>208</v>
+        <v>170</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="E11" s="10">
         <v>11</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>209</v>
+      <c r="F11" s="11">
+        <v>46245</v>
       </c>
       <c r="G11" s="10">
         <v>1972.66</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I11" s="10">
         <v>0</v>
@@ -1637,33 +1511,33 @@
         <v>46212</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A12" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>215</v>
+        <v>175</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>216</v>
+        <v>176</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E12" s="10">
         <v>12</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>217</v>
+      <c r="F12" s="11">
+        <v>46243</v>
       </c>
       <c r="G12" s="10">
         <v>1608.95</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I12" s="10">
         <v>0</v>
@@ -1675,7 +1549,7 @@
         <v>46212</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.15">
@@ -1683,25 +1557,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E13" s="10">
         <v>12</v>
       </c>
-      <c r="F13" s="10" t="s">
-        <v>63</v>
+      <c r="F13" s="11">
+        <v>46228</v>
       </c>
       <c r="G13" s="10">
         <v>600</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I13" s="10">
         <v>0</v>
@@ -1713,33 +1587,33 @@
         <v>46211</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A14" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="E14" s="10">
         <v>12</v>
       </c>
-      <c r="F14" s="10" t="s">
-        <v>85</v>
+      <c r="F14" s="11">
+        <v>46258</v>
       </c>
       <c r="G14" s="10">
         <v>999.91</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I14" s="10">
         <v>0</v>
@@ -1751,33 +1625,33 @@
         <v>46218</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A15" s="10" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>159</v>
+        <v>127</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>160</v>
+        <v>128</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E15" s="10">
         <v>12</v>
       </c>
-      <c r="F15" s="10" t="s">
-        <v>161</v>
+      <c r="F15" s="11">
+        <v>46311</v>
       </c>
       <c r="G15" s="10">
         <v>600</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I15" s="10">
         <v>0</v>
@@ -1789,33 +1663,33 @@
         <v>46205</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A16" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>121</v>
+        <v>96</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E16" s="10">
         <v>12</v>
       </c>
-      <c r="F16" s="10" t="s">
-        <v>25</v>
+      <c r="F16" s="11">
+        <v>46232</v>
       </c>
       <c r="G16" s="10">
         <v>650</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I16" s="10">
         <v>0</v>
@@ -1827,33 +1701,33 @@
         <v>46204</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A17" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>135</v>
+        <v>107</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>136</v>
+        <v>108</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E17" s="10">
         <v>12</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>55</v>
+      <c r="F17" s="11">
+        <v>46233</v>
       </c>
       <c r="G17" s="10">
         <v>500</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I17" s="10">
         <v>0</v>
@@ -1865,33 +1739,33 @@
         <v>46204</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A18" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>194</v>
+        <v>158</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>175</v>
+        <v>140</v>
       </c>
       <c r="E18" s="10">
         <v>12</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>55</v>
+      <c r="F18" s="11">
+        <v>46233</v>
       </c>
       <c r="G18" s="10">
         <v>500</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I18" s="10">
         <v>0</v>
@@ -1903,33 +1777,33 @@
         <v>46204</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A19" s="10" t="s">
-        <v>243</v>
+        <v>199</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>246</v>
+        <v>202</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>247</v>
+        <v>203</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E19" s="10">
         <v>11</v>
       </c>
-      <c r="F19" s="10" t="s">
-        <v>16</v>
+      <c r="F19" s="11">
+        <v>46214</v>
       </c>
       <c r="G19" s="10">
         <v>500</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I19" s="10">
         <v>7</v>
@@ -1941,7 +1815,7 @@
         <v>46204</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.15">
@@ -1949,25 +1823,25 @@
         <v>12</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E20" s="10">
         <v>12</v>
       </c>
-      <c r="F20" s="10" t="s">
-        <v>49</v>
+      <c r="F20" s="11">
+        <v>46231</v>
       </c>
       <c r="G20" s="10">
         <v>1999.6</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I20" s="10">
         <v>0</v>
@@ -1979,7 +1853,7 @@
         <v>46203</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.15">
@@ -1987,25 +1861,25 @@
         <v>12</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E21" s="10">
         <v>12</v>
       </c>
-      <c r="F21" s="10" t="s">
-        <v>55</v>
+      <c r="F21" s="11">
+        <v>46233</v>
       </c>
       <c r="G21" s="10">
         <v>800</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I21" s="10">
         <v>0</v>
@@ -2017,7 +1891,7 @@
         <v>46203</v>
       </c>
       <c r="L21" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.15">
@@ -2025,25 +1899,25 @@
         <v>12</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E22" s="10">
         <v>12</v>
       </c>
-      <c r="F22" s="10" t="s">
-        <v>58</v>
+      <c r="F22" s="11">
+        <v>46226</v>
       </c>
       <c r="G22" s="10">
         <v>1499.9</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I22" s="10">
         <v>0</v>
@@ -2055,7 +1929,7 @@
         <v>46203</v>
       </c>
       <c r="L22" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.15">
@@ -2063,25 +1937,25 @@
         <v>12</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="D23" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" s="10">
+        <v>0</v>
+      </c>
+      <c r="F23" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E23" s="10">
-        <v>0</v>
-      </c>
-      <c r="F23" s="10" t="s">
-        <v>20</v>
-      </c>
       <c r="G23" s="10">
         <v>0</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I23" s="10">
         <v>0</v>
@@ -2093,7 +1967,7 @@
         <v>46203</v>
       </c>
       <c r="L23" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.15">
@@ -2101,25 +1975,25 @@
         <v>12</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="E24" s="10">
         <v>12</v>
       </c>
-      <c r="F24" s="10" t="s">
-        <v>67</v>
+      <c r="F24" s="11">
+        <v>46225</v>
       </c>
       <c r="G24" s="10">
         <v>400</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I24" s="10">
         <v>0</v>
@@ -2131,33 +2005,33 @@
         <v>46203</v>
       </c>
       <c r="L24" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A25" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E25" s="10">
         <v>12</v>
       </c>
-      <c r="F25" s="10" t="s">
-        <v>71</v>
+      <c r="F25" s="11">
+        <v>46247</v>
       </c>
       <c r="G25" s="10">
         <v>500</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I25" s="10">
         <v>0</v>
@@ -2169,33 +2043,33 @@
         <v>46216</v>
       </c>
       <c r="L25" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A26" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E26" s="10">
         <v>12</v>
       </c>
-      <c r="F26" s="10" t="s">
-        <v>100</v>
+      <c r="F26" s="11">
+        <v>46239</v>
       </c>
       <c r="G26" s="10">
         <v>179.98</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I26" s="10">
         <v>0</v>
@@ -2207,33 +2081,33 @@
         <v>46209</v>
       </c>
       <c r="L26" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A27" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E27" s="10">
         <v>12</v>
       </c>
-      <c r="F27" s="10" t="s">
-        <v>63</v>
+      <c r="F27" s="11">
+        <v>46228</v>
       </c>
       <c r="G27" s="10">
         <v>500</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I27" s="10">
         <v>0</v>
@@ -2245,33 +2119,33 @@
         <v>46203</v>
       </c>
       <c r="L27" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A28" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>133</v>
+        <v>105</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>134</v>
+        <v>106</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="E28" s="10">
         <v>12</v>
       </c>
-      <c r="F28" s="10" t="s">
-        <v>55</v>
+      <c r="F28" s="11">
+        <v>46233</v>
       </c>
       <c r="G28" s="10">
         <v>1799.65</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I28" s="10">
         <v>0</v>
@@ -2283,33 +2157,33 @@
         <v>46203</v>
       </c>
       <c r="L28" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A29" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="E29" s="10">
         <v>12</v>
       </c>
-      <c r="F29" s="10" t="s">
-        <v>55</v>
+      <c r="F29" s="11">
+        <v>46233</v>
       </c>
       <c r="G29" s="10">
         <v>500</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I29" s="10">
         <v>0</v>
@@ -2321,33 +2195,33 @@
         <v>46203</v>
       </c>
       <c r="L29" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A30" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>141</v>
+        <v>113</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>142</v>
+        <v>114</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E30" s="10">
         <v>12</v>
       </c>
-      <c r="F30" s="10" t="s">
-        <v>25</v>
+      <c r="F30" s="11">
+        <v>46232</v>
       </c>
       <c r="G30" s="10">
         <v>941.28</v>
       </c>
       <c r="H30" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I30" s="10">
         <v>0</v>
@@ -2359,33 +2233,33 @@
         <v>46203</v>
       </c>
       <c r="L30" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A31" s="10" t="s">
-        <v>145</v>
+        <v>117</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>146</v>
+        <v>118</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E31" s="10">
         <v>12</v>
       </c>
-      <c r="F31" s="10" t="s">
-        <v>148</v>
+      <c r="F31" s="11">
+        <v>46019</v>
       </c>
       <c r="G31" s="10">
         <v>299.99</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I31" s="10">
         <v>202</v>
@@ -2397,33 +2271,33 @@
         <v>46203</v>
       </c>
       <c r="L31" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A32" s="10" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>154</v>
+        <v>124</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>155</v>
+        <v>125</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E32" s="10">
         <v>12</v>
       </c>
-      <c r="F32" s="10" t="s">
-        <v>156</v>
+      <c r="F32" s="11">
+        <v>46045</v>
       </c>
       <c r="G32" s="10">
         <v>936.73</v>
       </c>
       <c r="H32" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I32" s="10">
         <v>176</v>
@@ -2435,33 +2309,33 @@
         <v>46203</v>
       </c>
       <c r="L32" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A33" s="10" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>167</v>
+        <v>133</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>168</v>
+        <v>134</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E33" s="10">
         <v>18</v>
       </c>
-      <c r="F33" s="10" t="s">
-        <v>169</v>
+      <c r="F33" s="11">
+        <v>45991</v>
       </c>
       <c r="G33" s="10">
         <v>451.01</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I33" s="10">
         <v>230</v>
@@ -2473,33 +2347,33 @@
         <v>46203</v>
       </c>
       <c r="L33" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A34" s="10" t="s">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>173</v>
+        <v>138</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>174</v>
+        <v>139</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>175</v>
+        <v>140</v>
       </c>
       <c r="E34" s="10">
         <v>12</v>
       </c>
-      <c r="F34" s="10" t="s">
-        <v>55</v>
+      <c r="F34" s="11">
+        <v>46233</v>
       </c>
       <c r="G34" s="10">
         <v>1499.5</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I34" s="10">
         <v>0</v>
@@ -2511,33 +2385,33 @@
         <v>46203</v>
       </c>
       <c r="L34" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A35" s="10" t="s">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>176</v>
+        <v>141</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>177</v>
+        <v>142</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E35" s="10">
         <v>12</v>
       </c>
-      <c r="F35" s="10" t="s">
-        <v>115</v>
+      <c r="F35" s="11">
+        <v>46223</v>
       </c>
       <c r="G35" s="10">
         <v>999.98</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I35" s="10">
         <v>0</v>
@@ -2549,33 +2423,33 @@
         <v>46203</v>
       </c>
       <c r="L35" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A36" s="10" t="s">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>180</v>
+        <v>145</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>181</v>
+        <v>146</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E36" s="10">
         <v>12</v>
       </c>
-      <c r="F36" s="10" t="s">
-        <v>55</v>
+      <c r="F36" s="11">
+        <v>46233</v>
       </c>
       <c r="G36" s="10">
         <v>1199.8</v>
       </c>
       <c r="H36" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I36" s="10">
         <v>0</v>
@@ -2587,33 +2461,33 @@
         <v>46203</v>
       </c>
       <c r="L36" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A37" s="10" t="s">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>182</v>
+        <v>147</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>183</v>
+        <v>148</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>175</v>
+        <v>140</v>
       </c>
       <c r="E37" s="10">
         <v>12</v>
       </c>
-      <c r="F37" s="10" t="s">
-        <v>55</v>
+      <c r="F37" s="11">
+        <v>46233</v>
       </c>
       <c r="G37" s="10">
         <v>500</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I37" s="10">
         <v>0</v>
@@ -2625,33 +2499,33 @@
         <v>46203</v>
       </c>
       <c r="L37" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A38" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>190</v>
+        <v>154</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>191</v>
+        <v>155</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>192</v>
+        <v>156</v>
       </c>
       <c r="E38" s="10">
         <v>12</v>
       </c>
-      <c r="F38" s="10" t="s">
-        <v>21</v>
+      <c r="F38" s="11">
+        <v>46217</v>
       </c>
       <c r="G38" s="10">
         <v>1041.5</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I38" s="10">
         <v>4</v>
@@ -2663,33 +2537,33 @@
         <v>46203</v>
       </c>
       <c r="L38" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A39" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>200</v>
+        <v>163</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>201</v>
+        <v>164</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E39" s="10">
         <v>12</v>
       </c>
-      <c r="F39" s="10" t="s">
-        <v>55</v>
+      <c r="F39" s="11">
+        <v>46233</v>
       </c>
       <c r="G39" s="10">
         <v>700</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I39" s="10">
         <v>0</v>
@@ -2701,33 +2575,33 @@
         <v>46203</v>
       </c>
       <c r="L39" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A40" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>210</v>
+        <v>171</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>211</v>
+        <v>172</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="E40" s="10">
         <v>18</v>
       </c>
-      <c r="F40" s="10" t="s">
-        <v>212</v>
+      <c r="F40" s="11">
+        <v>46234</v>
       </c>
       <c r="G40" s="10">
         <v>951.99</v>
       </c>
       <c r="H40" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I40" s="10">
         <v>0</v>
@@ -2739,33 +2613,33 @@
         <v>46203</v>
       </c>
       <c r="L40" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A41" s="10" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>219</v>
+        <v>178</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>220</v>
+        <v>179</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E41" s="10">
         <v>12</v>
       </c>
-      <c r="F41" s="10" t="s">
-        <v>25</v>
+      <c r="F41" s="11">
+        <v>46232</v>
       </c>
       <c r="G41" s="10">
         <v>999.97</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I41" s="10">
         <v>0</v>
@@ -2777,33 +2651,33 @@
         <v>46203</v>
       </c>
       <c r="L41" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A42" s="10" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>226</v>
+        <v>184</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>224</v>
+        <v>183</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="E42" s="10">
         <v>12</v>
       </c>
-      <c r="F42" s="10" t="s">
-        <v>55</v>
+      <c r="F42" s="11">
+        <v>46233</v>
       </c>
       <c r="G42" s="10">
         <v>500</v>
       </c>
       <c r="H42" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I42" s="10">
         <v>0</v>
@@ -2815,33 +2689,33 @@
         <v>46203</v>
       </c>
       <c r="L42" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A43" s="10" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>228</v>
+        <v>186</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>229</v>
+        <v>187</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E43" s="10">
         <v>12</v>
       </c>
-      <c r="F43" s="10" t="s">
-        <v>45</v>
+      <c r="F43" s="11">
+        <v>46189</v>
       </c>
       <c r="G43" s="10">
         <v>100</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I43" s="10">
         <v>32</v>
@@ -2853,33 +2727,33 @@
         <v>46203</v>
       </c>
       <c r="L43" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A44" s="10" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>231</v>
+        <v>189</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>232</v>
+        <v>190</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="E44" s="10">
         <v>12</v>
       </c>
-      <c r="F44" s="10" t="s">
-        <v>55</v>
+      <c r="F44" s="11">
+        <v>46233</v>
       </c>
       <c r="G44" s="10">
         <v>999.94</v>
       </c>
       <c r="H44" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I44" s="10">
         <v>0</v>
@@ -2891,33 +2765,33 @@
         <v>46203</v>
       </c>
       <c r="L44" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A45" s="10" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>241</v>
+        <v>197</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>242</v>
+        <v>198</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E45" s="10">
         <v>12</v>
       </c>
-      <c r="F45" s="10" t="s">
-        <v>55</v>
+      <c r="F45" s="11">
+        <v>46233</v>
       </c>
       <c r="G45" s="10">
         <v>600</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I45" s="10">
         <v>0</v>
@@ -2929,33 +2803,33 @@
         <v>46203</v>
       </c>
       <c r="L45" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A46" s="10" t="s">
-        <v>243</v>
+        <v>199</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>244</v>
+        <v>200</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>245</v>
+        <v>201</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E46" s="10">
         <v>12</v>
       </c>
-      <c r="F46" s="10" t="s">
-        <v>40</v>
+      <c r="F46" s="11">
+        <v>46021</v>
       </c>
       <c r="G46" s="10">
         <v>144717.42000000001</v>
       </c>
       <c r="H46" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I46" s="10">
         <v>200</v>
@@ -2967,7 +2841,7 @@
         <v>46203</v>
       </c>
       <c r="L46" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.15">
@@ -2975,25 +2849,25 @@
         <v>12</v>
       </c>
       <c r="B47" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D47" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C47" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D47" s="10" t="s">
-        <v>24</v>
-      </c>
       <c r="E47" s="10">
         <v>12</v>
       </c>
-      <c r="F47" s="10" t="s">
-        <v>25</v>
+      <c r="F47" s="11">
+        <v>46232</v>
       </c>
       <c r="G47" s="10">
         <v>898.92</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I47" s="10">
         <v>0</v>
@@ -3005,7 +2879,7 @@
         <v>46200</v>
       </c>
       <c r="L47" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.15">
@@ -3013,25 +2887,25 @@
         <v>12</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E48" s="10">
         <v>12</v>
       </c>
-      <c r="F48" s="10" t="s">
-        <v>25</v>
+      <c r="F48" s="11">
+        <v>46232</v>
       </c>
       <c r="G48" s="10">
         <v>999.98</v>
       </c>
       <c r="H48" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I48" s="10">
         <v>0</v>
@@ -3043,33 +2917,33 @@
         <v>46200</v>
       </c>
       <c r="L48" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A49" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E49" s="10">
         <v>10</v>
       </c>
-      <c r="F49" s="10" t="s">
-        <v>112</v>
+      <c r="F49" s="11">
+        <v>46236</v>
       </c>
       <c r="G49" s="10">
         <v>950</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I49" s="10">
         <v>0</v>
@@ -3081,33 +2955,33 @@
         <v>46204</v>
       </c>
       <c r="L49" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A50" s="10" t="s">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>171</v>
+        <v>136</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>172</v>
+        <v>137</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="E50" s="10">
         <v>12</v>
       </c>
-      <c r="F50" s="10" t="s">
-        <v>63</v>
+      <c r="F50" s="11">
+        <v>46228</v>
       </c>
       <c r="G50" s="10">
         <v>500</v>
       </c>
       <c r="H50" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I50" s="10">
         <v>0</v>
@@ -3119,33 +2993,33 @@
         <v>46200</v>
       </c>
       <c r="L50" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A51" s="10" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>230</v>
+        <v>188</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>227</v>
+        <v>185</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="E51" s="10">
         <v>12</v>
       </c>
-      <c r="F51" s="10" t="s">
-        <v>35</v>
+      <c r="F51" s="11">
+        <v>46229</v>
       </c>
       <c r="G51" s="10">
         <v>999.93</v>
       </c>
       <c r="H51" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I51" s="10">
         <v>0</v>
@@ -3157,7 +3031,7 @@
         <v>46200</v>
       </c>
       <c r="L51" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.15">
@@ -3165,25 +3039,25 @@
         <v>12</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E52" s="10">
         <v>12</v>
       </c>
-      <c r="F52" s="10" t="s">
-        <v>35</v>
+      <c r="F52" s="11">
+        <v>46229</v>
       </c>
       <c r="G52" s="10">
         <v>2600.1</v>
       </c>
       <c r="H52" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I52" s="10">
         <v>0</v>
@@ -3195,33 +3069,33 @@
         <v>46199</v>
       </c>
       <c r="L52" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A53" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>137</v>
+        <v>109</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>138</v>
+        <v>110</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="E53" s="10">
         <v>12</v>
       </c>
-      <c r="F53" s="10" t="s">
-        <v>55</v>
+      <c r="F53" s="11">
+        <v>46233</v>
       </c>
       <c r="G53" s="10">
         <v>999.94</v>
       </c>
       <c r="H53" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I53" s="10">
         <v>0</v>
@@ -3233,33 +3107,33 @@
         <v>46199</v>
       </c>
       <c r="L53" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A54" s="10" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>162</v>
+        <v>129</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>163</v>
+        <v>130</v>
       </c>
       <c r="D54" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E54" s="10">
         <v>12</v>
       </c>
-      <c r="F54" s="10" t="s">
-        <v>63</v>
+      <c r="F54" s="11">
+        <v>46228</v>
       </c>
       <c r="G54" s="10">
         <v>35</v>
       </c>
       <c r="H54" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I54" s="10">
         <v>0</v>
@@ -3271,33 +3145,33 @@
         <v>46199</v>
       </c>
       <c r="L54" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A55" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>198</v>
+        <v>161</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>199</v>
+        <v>162</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E55" s="10">
         <v>12</v>
       </c>
-      <c r="F55" s="10" t="s">
-        <v>63</v>
+      <c r="F55" s="11">
+        <v>46228</v>
       </c>
       <c r="G55" s="10">
         <v>999.98</v>
       </c>
       <c r="H55" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I55" s="10">
         <v>0</v>
@@ -3309,33 +3183,33 @@
         <v>46199</v>
       </c>
       <c r="L55" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A56" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>202</v>
+        <v>165</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>203</v>
+        <v>166</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E56" s="10">
         <v>16</v>
       </c>
-      <c r="F56" s="10" t="s">
-        <v>35</v>
+      <c r="F56" s="11">
+        <v>46229</v>
       </c>
       <c r="G56" s="10">
         <v>620</v>
       </c>
       <c r="H56" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I56" s="10">
         <v>0</v>
@@ -3347,33 +3221,33 @@
         <v>46199</v>
       </c>
       <c r="L56" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A57" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>204</v>
+        <v>167</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>205</v>
+        <v>168</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E57" s="10">
         <v>24</v>
       </c>
-      <c r="F57" s="10" t="s">
-        <v>206</v>
+      <c r="F57" s="11">
+        <v>46230</v>
       </c>
       <c r="G57" s="10">
         <v>505</v>
       </c>
       <c r="H57" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I57" s="10">
         <v>0</v>
@@ -3385,33 +3259,33 @@
         <v>46199</v>
       </c>
       <c r="L57" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A58" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>213</v>
+        <v>173</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>214</v>
+        <v>174</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="E58" s="10">
         <v>12</v>
       </c>
-      <c r="F58" s="10" t="s">
-        <v>206</v>
+      <c r="F58" s="11">
+        <v>46230</v>
       </c>
       <c r="G58" s="10">
         <v>999.91</v>
       </c>
       <c r="H58" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I58" s="10">
         <v>0</v>
@@ -3423,33 +3297,33 @@
         <v>46199</v>
       </c>
       <c r="L58" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A59" s="10" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>233</v>
+        <v>191</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>234</v>
+        <v>192</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E59" s="10">
         <v>12</v>
       </c>
-      <c r="F59" s="10" t="s">
-        <v>235</v>
+      <c r="F59" s="11">
+        <v>46108</v>
       </c>
       <c r="G59" s="10">
         <v>919.99</v>
       </c>
       <c r="H59" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I59" s="10">
         <v>113</v>
@@ -3461,7 +3335,7 @@
         <v>46199</v>
       </c>
       <c r="L59" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.15">
@@ -3469,25 +3343,25 @@
         <v>12</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E60" s="10">
         <v>12</v>
       </c>
-      <c r="F60" s="10" t="s">
-        <v>44</v>
+      <c r="F60" s="11">
+        <v>45894</v>
       </c>
       <c r="G60" s="10">
         <v>449.99</v>
       </c>
       <c r="H60" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I60" s="10">
         <v>327</v>
@@ -3499,33 +3373,33 @@
         <v>46197</v>
       </c>
       <c r="L60" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A61" s="10" t="s">
-        <v>243</v>
+        <v>199</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>248</v>
+        <v>204</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>249</v>
+        <v>205</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="E61" s="10">
         <v>12</v>
       </c>
-      <c r="F61" s="10" t="s">
-        <v>88</v>
+      <c r="F61" s="11">
+        <v>46227</v>
       </c>
       <c r="G61" s="10">
         <v>700</v>
       </c>
       <c r="H61" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I61" s="10">
         <v>0</v>
@@ -3537,7 +3411,7 @@
         <v>46197</v>
       </c>
       <c r="L61" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.15">
@@ -3556,14 +3430,14 @@
       <c r="E62" s="10">
         <v>16</v>
       </c>
-      <c r="F62" s="10" t="s">
-        <v>16</v>
+      <c r="F62" s="11">
+        <v>46214</v>
       </c>
       <c r="G62" s="10">
         <v>572</v>
       </c>
       <c r="H62" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I62" s="10">
         <v>7</v>
@@ -3575,33 +3449,33 @@
         <v>46196</v>
       </c>
       <c r="L62" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A63" s="10" t="s">
-        <v>187</v>
+        <v>151</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>188</v>
+        <v>152</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>189</v>
+        <v>153</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E63" s="10">
         <v>6</v>
       </c>
-      <c r="F63" s="10" t="s">
-        <v>58</v>
+      <c r="F63" s="11">
+        <v>46226</v>
       </c>
       <c r="G63" s="10">
         <v>1674.9</v>
       </c>
       <c r="H63" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I63" s="10">
         <v>0</v>
@@ -3613,33 +3487,33 @@
         <v>46196</v>
       </c>
       <c r="L63" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A64" s="10" t="s">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>178</v>
+        <v>143</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>179</v>
+        <v>144</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E64" s="10">
         <v>12</v>
       </c>
-      <c r="F64" s="10" t="s">
-        <v>67</v>
+      <c r="F64" s="11">
+        <v>46225</v>
       </c>
       <c r="G64" s="10">
         <v>886.8</v>
       </c>
       <c r="H64" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I64" s="10">
         <v>0</v>
@@ -3651,33 +3525,33 @@
         <v>46195</v>
       </c>
       <c r="L64" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A65" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B65" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B65" s="10" t="s">
-        <v>86</v>
-      </c>
       <c r="C65" s="10" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E65" s="10">
         <v>12</v>
       </c>
-      <c r="F65" s="10" t="s">
-        <v>88</v>
+      <c r="F65" s="11">
+        <v>46227</v>
       </c>
       <c r="G65" s="10">
         <v>999.92</v>
       </c>
       <c r="H65" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I65" s="10">
         <v>0</v>
@@ -3689,33 +3563,33 @@
         <v>46203</v>
       </c>
       <c r="L65" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A66" s="10" t="s">
-        <v>218</v>
+        <v>177</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>238</v>
+        <v>195</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>239</v>
+        <v>196</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E66" s="10">
         <v>12</v>
       </c>
-      <c r="F66" s="10" t="s">
-        <v>240</v>
+      <c r="F66" s="11">
+        <v>45945</v>
       </c>
       <c r="G66" s="10">
         <v>1229.96</v>
       </c>
       <c r="H66" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I66" s="10">
         <v>276</v>
@@ -3727,33 +3601,33 @@
         <v>46190</v>
       </c>
       <c r="L66" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A67" s="10" t="s">
-        <v>145</v>
+        <v>117</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>149</v>
+        <v>120</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>150</v>
+        <v>121</v>
       </c>
       <c r="D67" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E67" s="10">
         <v>12</v>
       </c>
-      <c r="F67" s="10" t="s">
-        <v>151</v>
+      <c r="F67" s="11">
+        <v>46219</v>
       </c>
       <c r="G67" s="10">
         <v>1466.63</v>
       </c>
       <c r="H67" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I67" s="10">
         <v>2</v>
@@ -3765,33 +3639,33 @@
         <v>46189</v>
       </c>
       <c r="L67" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A68" s="10" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>157</v>
+        <v>126</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E68" s="10">
         <v>5</v>
       </c>
-      <c r="F68" s="10" t="s">
-        <v>158</v>
+      <c r="F68" s="11">
+        <v>46208</v>
       </c>
       <c r="G68" s="10">
         <v>999.99</v>
       </c>
       <c r="H68" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I68" s="10">
         <v>13</v>
@@ -3803,33 +3677,33 @@
         <v>46178</v>
       </c>
       <c r="L68" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A69" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>130</v>
+        <v>103</v>
       </c>
       <c r="C69" s="10" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="E69" s="10">
         <v>12</v>
       </c>
-      <c r="F69" s="10" t="s">
-        <v>132</v>
+      <c r="F69" s="11">
+        <v>46136</v>
       </c>
       <c r="G69" s="10">
         <v>2199.6</v>
       </c>
       <c r="H69" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I69" s="10">
         <v>85</v>
@@ -3841,33 +3715,33 @@
         <v>46175</v>
       </c>
       <c r="L69" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A70" s="10" t="s">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>184</v>
+        <v>149</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>185</v>
+        <v>150</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E70" s="10">
         <v>12</v>
       </c>
-      <c r="F70" s="10" t="s">
-        <v>186</v>
+      <c r="F70" s="11">
+        <v>46201</v>
       </c>
       <c r="G70" s="10">
         <v>22000.99</v>
       </c>
       <c r="H70" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I70" s="10">
         <v>20</v>
@@ -3879,33 +3753,33 @@
         <v>46170</v>
       </c>
       <c r="L70" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A71" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>127</v>
+        <v>101</v>
       </c>
       <c r="C71" s="10" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E71" s="10">
         <v>12</v>
       </c>
-      <c r="F71" s="10" t="s">
-        <v>129</v>
+      <c r="F71" s="11">
+        <v>46192</v>
       </c>
       <c r="G71" s="10">
         <v>1199.95</v>
       </c>
       <c r="H71" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I71" s="10">
         <v>29</v>
@@ -3917,33 +3791,33 @@
         <v>46161</v>
       </c>
       <c r="L71" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A72" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E72" s="10">
         <v>12</v>
       </c>
-      <c r="F72" s="10" t="s">
-        <v>79</v>
+      <c r="F72" s="11">
+        <v>45746</v>
       </c>
       <c r="G72" s="10">
         <v>54896.28</v>
       </c>
       <c r="H72" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I72" s="10">
         <v>475</v>
@@ -3955,33 +3829,33 @@
         <v>46203</v>
       </c>
       <c r="L72" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A73" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>122</v>
+        <v>97</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>123</v>
+        <v>98</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E73" s="10">
         <v>12</v>
       </c>
-      <c r="F73" s="10" t="s">
-        <v>124</v>
+      <c r="F73" s="11">
+        <v>46060</v>
       </c>
       <c r="G73" s="10">
         <v>1199.8499999999999</v>
       </c>
       <c r="H73" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I73" s="10">
         <v>161</v>
@@ -3993,33 +3867,33 @@
         <v>46084</v>
       </c>
       <c r="L73" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A74" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="E74" s="10">
         <v>11</v>
       </c>
-      <c r="F74" s="10" t="s">
-        <v>93</v>
+      <c r="F74" s="11">
+        <v>45758</v>
       </c>
       <c r="G74" s="10">
         <v>3178.1</v>
       </c>
       <c r="H74" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I74" s="10">
         <v>463</v>
@@ -4031,7 +3905,7 @@
         <v>46203</v>
       </c>
       <c r="L74" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.15">
@@ -4039,25 +3913,25 @@
         <v>12</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E75" s="10">
         <v>12</v>
       </c>
-      <c r="F75" s="10" t="s">
-        <v>52</v>
+      <c r="F75" s="11">
+        <v>45897</v>
       </c>
       <c r="G75" s="10">
         <v>12532.5</v>
       </c>
       <c r="H75" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I75" s="10">
         <v>324</v>
@@ -4069,33 +3943,33 @@
         <v>46048</v>
       </c>
       <c r="L75" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A76" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="E76" s="10">
         <v>6</v>
       </c>
-      <c r="F76" s="10" t="s">
-        <v>25</v>
+      <c r="F76" s="11">
+        <v>46232</v>
       </c>
       <c r="G76" s="10">
         <v>1682.3</v>
       </c>
       <c r="H76" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I76" s="10">
         <v>0</v>
@@ -4107,33 +3981,33 @@
         <v>46203</v>
       </c>
       <c r="L76" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A77" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="C77" s="10" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E77" s="10">
         <v>12</v>
       </c>
-      <c r="F77" s="10" t="s">
-        <v>55</v>
+      <c r="F77" s="11">
+        <v>46233</v>
       </c>
       <c r="G77" s="10">
         <v>2433.9</v>
       </c>
       <c r="H77" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I77" s="10">
         <v>0</v>
@@ -4145,33 +4019,33 @@
         <v>46203</v>
       </c>
       <c r="L77" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A78" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E78" s="10">
         <v>16</v>
       </c>
-      <c r="F78" s="10" t="s">
-        <v>55</v>
+      <c r="F78" s="11">
+        <v>46233</v>
       </c>
       <c r="G78" s="10">
         <v>920</v>
       </c>
       <c r="H78" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I78" s="10">
         <v>0</v>
@@ -4183,33 +4057,33 @@
         <v>46203</v>
       </c>
       <c r="L78" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A79" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="D79" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E79" s="10">
         <v>12</v>
       </c>
-      <c r="F79" s="10" t="s">
-        <v>55</v>
+      <c r="F79" s="11">
+        <v>46233</v>
       </c>
       <c r="G79" s="10">
         <v>46963.45</v>
       </c>
       <c r="H79" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I79" s="10">
         <v>0</v>
@@ -4221,33 +4095,33 @@
         <v>46203</v>
       </c>
       <c r="L79" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A80" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E80" s="10">
         <v>12</v>
       </c>
-      <c r="F80" s="10" t="s">
-        <v>16</v>
+      <c r="F80" s="11">
+        <v>46214</v>
       </c>
       <c r="G80" s="10">
         <v>35352.129999999997</v>
       </c>
       <c r="H80" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I80" s="10">
         <v>7</v>
@@ -4259,33 +4133,33 @@
         <v>46200</v>
       </c>
       <c r="L80" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A81" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="C81" s="10" t="s">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="E81" s="10">
         <v>12</v>
       </c>
-      <c r="F81" s="10" t="s">
-        <v>63</v>
+      <c r="F81" s="11">
+        <v>46228</v>
       </c>
       <c r="G81" s="10">
         <v>999.91</v>
       </c>
       <c r="H81" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I81" s="10">
         <v>0</v>
@@ -4297,33 +4171,33 @@
         <v>46199</v>
       </c>
       <c r="L81" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A82" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B82" s="10" t="s">
-        <v>106</v>
+        <v>85</v>
       </c>
       <c r="C82" s="10" t="s">
-        <v>107</v>
+        <v>86</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="E82" s="10">
         <v>12</v>
       </c>
-      <c r="F82" s="10" t="s">
-        <v>109</v>
+      <c r="F82" s="11">
+        <v>46222</v>
       </c>
       <c r="G82" s="10">
         <v>685.15</v>
       </c>
       <c r="H82" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I82" s="10">
         <v>0</v>
@@ -4335,33 +4209,33 @@
         <v>46193</v>
       </c>
       <c r="L82" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A83" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="C83" s="10" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E83" s="10">
         <v>12</v>
       </c>
-      <c r="F83" s="10" t="s">
-        <v>67</v>
+      <c r="F83" s="11">
+        <v>46225</v>
       </c>
       <c r="G83" s="10">
         <v>1155.28</v>
       </c>
       <c r="H83" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I83" s="10">
         <v>0</v>
@@ -4373,33 +4247,33 @@
         <v>46193</v>
       </c>
       <c r="L83" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A84" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="C84" s="10" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E84" s="10">
         <v>12</v>
       </c>
-      <c r="F84" s="10" t="s">
-        <v>115</v>
+      <c r="F84" s="11">
+        <v>46223</v>
       </c>
       <c r="G84" s="10">
         <v>706</v>
       </c>
       <c r="H84" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I84" s="10">
         <v>0</v>
@@ -4411,33 +4285,33 @@
         <v>46193</v>
       </c>
       <c r="L84" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A85" s="10" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E85" s="10">
         <v>12</v>
       </c>
-      <c r="F85" s="10" t="s">
-        <v>63</v>
+      <c r="F85" s="11">
+        <v>46228</v>
       </c>
       <c r="G85" s="10">
         <v>1499.6</v>
       </c>
       <c r="H85" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I85" s="10">
         <v>0</v>
@@ -4449,22 +4323,46 @@
         <v>46193</v>
       </c>
       <c r="L85" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="86" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A86"/>
-      <c r="B86"/>
-      <c r="C86"/>
-      <c r="D86"/>
-      <c r="E86"/>
-      <c r="F86"/>
-      <c r="G86"/>
-      <c r="H86"/>
-      <c r="I86"/>
-      <c r="J86"/>
-      <c r="K86"/>
-      <c r="L86"/>
+      <c r="A86" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B86" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="C86" t="s">
+        <v>150</v>
+      </c>
+      <c r="D86">
+        <v>1</v>
+      </c>
+      <c r="E86" s="13">
+        <v>12</v>
+      </c>
+      <c r="F86" s="11">
+        <v>46261</v>
+      </c>
+      <c r="G86" s="13">
+        <v>1500</v>
+      </c>
+      <c r="H86" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="I86" s="13">
+        <v>0</v>
+      </c>
+      <c r="J86" s="13">
+        <v>21000</v>
+      </c>
+      <c r="K86" s="14">
+        <v>46230</v>
+      </c>
+      <c r="L86" s="10" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="87" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A87"/>
@@ -6154,7 +6052,7 @@
   </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.59055118110236227" bottom="0.39370078740157483" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="46" orientation="landscape"/>
+  <pageSetup paperSize="9" scale="46" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>